<commit_message>
docs: set financial model defaults to the bootstrapped plan
Payroll 2L/3L/5L, ads 25k/1L/2L, champions on commission only.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RiTsdM6K46HbTGVR4HVBpm
</commit_message>
<xml_diff>
--- a/docs/gtm/Decibyl-Financial-Model.xlsx
+++ b/docs/gtm/Decibyl-Financial-Model.xlsx
@@ -1442,11 +1442,11 @@
         </is>
       </c>
       <c r="B73" s="11" t="n">
-        <v>50000</v>
+        <v>25000</v>
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Assumption</t>
+          <t>Bootstrapped plan, 14 Sept: step up only after CAC and conversion are measured</t>
         </is>
       </c>
     </row>
@@ -1457,9 +1457,13 @@
         </is>
       </c>
       <c r="B74" s="11" t="n">
-        <v>150000</v>
-      </c>
-      <c r="D74" s="9" t="inlineStr"/>
+        <v>100000</v>
+      </c>
+      <c r="D74" s="9" t="inlineStr">
+        <is>
+          <t>Funded from revenue</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
@@ -1468,7 +1472,7 @@
         </is>
       </c>
       <c r="B75" s="11" t="n">
-        <v>300000</v>
+        <v>200000</v>
       </c>
       <c r="D75" s="9" t="inlineStr"/>
     </row>
@@ -1550,11 +1554,11 @@
         </is>
       </c>
       <c r="B81" s="11" t="n">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>₹15k to ₹25k</t>
+          <t>Bootstrapped: commission only; ₹15k to ₹25k once revenue supports it</t>
         </is>
       </c>
     </row>
@@ -1713,11 +1717,11 @@
         </is>
       </c>
       <c r="B94" s="11" t="n">
-        <v>300000</v>
+        <v>200000</v>
       </c>
       <c r="D94" s="9" t="inlineStr">
         <is>
-          <t>Assumption: 2 engineers + founder minimal; edit</t>
+          <t>Bootstrapped: founder + 1 engineer</t>
         </is>
       </c>
     </row>
@@ -1728,9 +1732,13 @@
         </is>
       </c>
       <c r="B95" s="11" t="n">
-        <v>450000</v>
-      </c>
-      <c r="D95" s="9" t="inlineStr"/>
+        <v>300000</v>
+      </c>
+      <c r="D95" s="9" t="inlineStr">
+        <is>
+          <t>Second engineer once EBITDA is positive</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
@@ -1739,7 +1747,7 @@
         </is>
       </c>
       <c r="B96" s="11" t="n">
-        <v>700000</v>
+        <v>500000</v>
       </c>
       <c r="D96" s="9" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
feat: site pricing on the shipped credits model, with the full rate card
Plans, credits, caps, voice rates, top-up packs, overage rule and the six
Free steps are copied from what the platform sells (LADDER_SEED,
plan_limits.SEED, EVENT_CREDITS, topup_packs, bundles). Every event's
credit price is published; Natural and Premium are shown as itemised.
Jobs and verticals now recommend Business as the first voice plan.
Financial model rebuilt on the shipped ladder (0 formula errors); spec
carries an as-shipped reconciliation banner.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RiTsdM6K46HbTGVR4HVBpm
</commit_message>
<xml_diff>
--- a/docs/gtm/Decibyl-Financial-Model.xlsx
+++ b/docs/gtm/Decibyl-Financial-Model.xlsx
@@ -651,7 +651,7 @@
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Pricing decision, 14 Sept</t>
+          <t>As shipped 14 Sept: subscription_plans.py LADDER_SEED</t>
         </is>
       </c>
     </row>
@@ -752,7 +752,7 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>Pricing decision, 14 Sept</t>
+          <t>As shipped 14 Sept: subscription_plans.py LADDER_SEED</t>
         </is>
       </c>
     </row>
@@ -763,7 +763,7 @@
         </is>
       </c>
       <c r="B24" s="8" t="n">
-        <v>5000</v>
+        <v>6000</v>
       </c>
       <c r="D24" s="9" t="inlineStr"/>
     </row>
@@ -849,11 +849,11 @@
         </is>
       </c>
       <c r="B30" s="11" t="n">
-        <v>7999</v>
+        <v>9999</v>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>Pricing decision, 14 Sept</t>
+          <t>As shipped 14 Sept: subscription_plans.py LADDER_SEED</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="B31" s="8" t="n">
-        <v>15000</v>
+        <v>25000</v>
       </c>
       <c r="D31" s="9" t="inlineStr"/>
     </row>
@@ -954,7 +954,7 @@
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>Pricing decision, 14 Sept</t>
+          <t>As shipped 14 Sept: subscription_plans.py LADDER_SEED</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
         </is>
       </c>
       <c r="B38" s="8" t="n">
-        <v>40000</v>
+        <v>60000</v>
       </c>
       <c r="D38" s="9" t="inlineStr"/>
     </row>
@@ -1073,11 +1073,11 @@
         </is>
       </c>
       <c r="B46" s="8" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>Growth 11, Scale 10; blended here at 12 for a conservative COGS</t>
+          <t>Shipped 14 Sept (KAN-47 PR #273): 13 Business, 12 Growth, 11 Scale; blended at 13 for a conservative COGS</t>
         </is>
       </c>
     </row>

</xml_diff>